<commit_message>
Update Brian Summa's content from his 2026 CV
- Papers: full author lists; HistoCAM final title (Nature Communications);
  NeurIPS, ICML, and EMNLP 2026 acceptances; VIS 2024 Best Paper and
  BOE Editor's Pick awards; Tulane-era papers, abstracts, and posters
  from 2016 on (86 publications in total)
- Grants: exact titles, roles, and amounts for ARPA-H, NIH, and DOE;
  add GoMed, QuBBD, EAGER, CRII, and the NSF IUCRC planning grant
- People: Kimberly Ashman as research staff; graduation years and
  co-advisors for Brian's PhD alumni; updated research interests
- News: VIS 2024 Best Paper, 2026 acceptances, HistoCAM, IEEE CS
  Distinguished Service Award, 2025 awards, Aug 2026 webinar talk
- Grants sentence names each funder once (NSF/NIH counts as both)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nn3skUUzonfjGHPGXscANL
</commit_message>
<xml_diff>
--- a/content/hcc-content.xlsx
+++ b/content/hcc-content.xlsx
@@ -771,7 +771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Data visualization; Computer graphics; Topological data analysis; Image processing; Large data</t>
+          <t>Visualization; Topological data analysis; Image processing; Applied machine learning; Digital pathology</t>
         </is>
       </c>
     </row>
@@ -1107,6 +1107,36 @@
       </c>
       <c r="M5" s="3" t="n"/>
       <c r="N5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Kimberly Ashman</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Research Staff</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>images/people/kimberly-ashman.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O5"/>
@@ -1726,7 +1756,9 @@
       </c>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
+      <c r="G12" s="3" t="n">
+        <v>2024</v>
+      </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Accelya Group</t>
@@ -1773,12 +1805,14 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Brian</t>
+          <t>Brian, J. Quincy Brown</t>
         </is>
       </c>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
+      <c r="G13" s="3" t="n">
+        <v>2022</v>
+      </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
           <t>FDA</t>
@@ -1817,15 +1851,17 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Brian</t>
+          <t>Brian, J. Quincy Brown</t>
         </is>
       </c>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
+      <c r="G14" s="3" t="n">
+        <v>2022</v>
+      </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>New York Yankees Sports Analytics</t>
+          <t>research staff in the group, after New York Yankees Sports Analytics</t>
         </is>
       </c>
       <c r="I14" s="3" t="n"/>
@@ -1867,7 +1903,7 @@
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
@@ -3400,7 +3436,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>MAGIC-SCAN; PathCAM; Medical image processing</t>
+          <t>MAGIC-SCAN; PathCAM; HistoCAM; Medical image processing</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3456,7 +3492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T64"/>
+  <dimension ref="A1:T87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4626,7 +4662,11 @@
       <c r="N17" s="3" t="n"/>
       <c r="O17" s="3" t="n"/>
       <c r="P17" s="3" t="n"/>
-      <c r="Q17" s="3" t="n"/>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>Best Paper Award, IEEE VIS 2024</t>
+        </is>
+      </c>
       <c r="R17" s="3" t="n"/>
       <c r="S17" s="3" t="n"/>
       <c r="T17" s="3" t="n"/>
@@ -5550,7 +5590,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Workshop Paper</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -5593,12 +5633,12 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>arXiv</t>
+          <t>TopoInVis</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Workshop Paper</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -5811,7 +5851,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Thomas Richard; Yan Chastagnier; Vivien Szabo; Kevin Chalard; Brian Summa; Jean-Marc Thiery; Tamy Boubekeur; Noura Faraj</t>
+          <t>Thibault Richard; Noura Faraj; Yan Chastagnier; Vivien Szabo; Kevin Chalard; Brian Summa; Jean-Marc Thiery; Tamy Boubekeur</t>
         </is>
       </c>
       <c r="I37" s="3" t="n"/>
@@ -5892,12 +5932,12 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>arXiv</t>
+          <t>EMNLP</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -6021,12 +6061,12 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>arXiv</t>
+          <t>ICML</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -6160,7 +6200,7 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>Kimberly Ashman; Huimin Zhuge; E. Shanley; Sharon Fox; S. Halat; Andrew Sholl; Brian Summa; J. Quincy Brown</t>
+          <t>Kimberly Ashman; Huimin Zhuge; Erin Shanley; Sharon Fox; Shams Halat; Andrew Sholl; Brian Summa; J. Quincy Brown</t>
         </is>
       </c>
       <c r="I45" s="3" t="n"/>
@@ -6193,12 +6233,12 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>arXiv</t>
+          <t>NeurIPS</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -6233,7 +6273,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Ambient, Real-Time Digitization and Datafication of Glass Slide Microscopy towards AI-at-the-Microscope</t>
+          <t>HistoCAM: Datafying the Diagnostic Process and Enabling AI-at-the-Microscope via Ambient, Real-Time Digitization of Glass Slide Microscopy</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
@@ -6251,7 +6291,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>Cooper Maira; Max S. Cooper; Kimberly Ashman; Andrew B. Sholl; Sharon E. Fox; S. Halat; D. Manthey; et al.; Brian Summa</t>
+          <t>Cooper Maira; Max Cooper; Kimberly Ashman; Andrew Sholl; Sharon Fox; Shams Halat; David Manthey; Roni Choudhury; Jonathan Sears; Carola Wenk; J. Quincy Brown; Brian Summa</t>
         </is>
       </c>
       <c r="I47" s="3" t="n"/>
@@ -6291,7 +6331,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>I. Bozic; G. J. Kobza; L. E. Boudreaux; D. A. Lucia; Emily Ribando-Gros; Kimberly Ashman; et al.; Brian Summa</t>
+          <t>Ivana Bozic; Grant J. Kobza; Lauren E. Boudreaux; Dylan A. Lucia; Emily Ribando-Gros; Kimberly Ashman; Brian Summa; J. Quincy Brown</t>
         </is>
       </c>
       <c r="I48" s="3" t="n"/>
@@ -6331,7 +6371,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>Syed Fahim Ahmed; Gnanesh Rasineni; Florian Koehler; Abu Zahid Bin Aziz; M. Wang; Attila Gyulassy; et al.; Brian Summa</t>
+          <t>Syed Fahim Ahmed; Gnanesh Rasineni; Florian Koehler; Abu Zahid Bin Aziz; Mei Wang; Attila Gyulassy; Brian Summa; J. Quincy Brown; Valerio Pascucci; Shireen Y. Elhabian</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -6375,7 +6415,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>I. Bozic; C. W. Simmons; D. A. Lucia; R. C. Todaro; Brian Summa; P. Kner; J. Quincy Brown</t>
+          <t>Ivana Bozic; Christopher W. Simmons; Dylan A. Lucia; Richard C. Todaro; Brian Summa; Peter Kner; J. Quincy Brown</t>
         </is>
       </c>
       <c r="I50" s="3" t="n"/>
@@ -6415,7 +6455,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>Max S. Cooper; Cooper Maira; Kimberly Ashman; Andrew B. Sholl; Sharon E. Fox; Carola Wenk; Brian Summa; et al.</t>
+          <t>Max Cooper; Cooper Maira; Kimberly Ashman; Andrew Sholl; Sharon Fox; Carola Wenk; Brian Summa; J. Quincy Brown</t>
         </is>
       </c>
       <c r="I51" s="3" t="n"/>
@@ -6445,7 +6485,7 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>US Patent App.</t>
+          <t>US Patent</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -6463,7 +6503,7 @@
       <c r="Q52" s="3" t="n"/>
       <c r="T52" s="3" t="inlineStr">
         <is>
-          <t>Application 19/375,404 (2026): https://patents.google.com/?q=19%2F375%2C404; Application 18/279,171 (2024): https://patents.google.com/?q=18%2F279%2C171</t>
+          <t>Google Patents: https://patents.google.com/patent/US20260057632A1/en</t>
         </is>
       </c>
     </row>
@@ -6499,7 +6539,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>Max S. Cooper; Cooper Maira; Kimberly Ashman; S. Halat; Andrew B. Sholl; Carola Wenk; Sharon E. Fox; et al.; Brian Summa</t>
+          <t>Max Cooper; Cooper Maira; Kimberly Ashman; Shams Halat; Andrew Sholl; Carola Wenk; Sharon Fox; Brian Summa; J. Quincy Brown</t>
         </is>
       </c>
       <c r="I53" s="3" t="n"/>
@@ -6539,7 +6579,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>Max S. Cooper; Kimberly Ashman; Cooper Maira; S. Halat; Andrew B. Sholl; Carola Wenk; Sharon E. Fox; et al.; Brian Summa</t>
+          <t>Max S. Cooper; Kimberly Ashman; Cooper Maira; Shams Halat; Andrew Sholl; Carola Wenk; Sharon Fox; Brian Summa; J. Quincy Brown</t>
         </is>
       </c>
       <c r="I54" s="3" t="n"/>
@@ -6579,12 +6619,16 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>Huimin Zhuge; Brian Summa; J. Hamm; J. Quincy Brown</t>
+          <t>Huimin Zhuge; Brian Summa; Jihun Hamm; J. Quincy Brown</t>
         </is>
       </c>
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="3" t="n"/>
-      <c r="Q55" s="3" t="n"/>
+      <c r="Q55" s="3" t="inlineStr">
+        <is>
+          <t>Editor's Pick</t>
+        </is>
+      </c>
       <c r="T55" s="3" t="inlineStr">
         <is>
           <t>PubMed: https://pubmed.ncbi.nlm.nih.gov/35003850/</t>
@@ -6663,7 +6707,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>Duong Hoang; Brian Summa; Harsh Bhatia; Peter Lindstrom; Pavol Klacansky; Will Usher; Peer-Timo Bremer; Valerio Pascucci</t>
+          <t>Duong Hoang; Brian Summa; Pavol Klacansky; Will Usher; Harsh Bhatia; Peter Lindstrom; Peer-Timo Bremer; Valerio Pascucci</t>
         </is>
       </c>
       <c r="I57" s="3" t="n"/>
@@ -6982,6 +7026,821 @@
       <c r="J64" s="3" t="n"/>
       <c r="Q64" s="3" t="n"/>
       <c r="T64" s="3" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Brian, Fangzheng</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Behavior-Discriminative Reward Shaping for Reward-Robust Reinforcement Learning</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>NeurIPS</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Full Paper</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Zixuan Liu; Fangzheng Wu; Brian Summa; Zizhan Zheng</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Topological Guided Detection of Extreme Wind Phenomena: Implications for Wind Energy</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>EnergyVis</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Workshop Paper</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Yu Qin; Graham Johnson; Brian Summa</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>PathCAM: Pathology Computer Assisted Microscope for Multiscale Expert-in-the-Loop Digital Pathology</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>SPIE</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>J. Quincy Brown; Kimberly Ashman; Max Cooper; Huimin Zhuge; Sharon E. Fox; Jonathan I. Epstein; Carola Wenk; Brian Summa</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Multi-Organ COVID-19 Autopsy Findings Using Three-Dimensional Virtual Histology Imaging</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Optica Biophotonics</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Guang Li; Sharon Fox; Huimin Zhuge; Brian Summa; Bihe Hu; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Reconstructing a Multiscale Digital Record of Clinical Pathology Slide Review Using Onboard-Cameras</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Optica Biophotonics</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Kimberly Ashman; Max S. Cooper; Sharon Fox; Brian Summa; J. Quincy Brown</t>
+        </is>
+      </c>
+      <c r="T69" s="3" t="inlineStr">
+        <is>
+          <t>Optica: https://opg.optica.org/abstract.cfm?uri=Microscopy-2022-MW4A.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Visualizing Analog and Digital Diagnostic Provenance in Pathology</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Optica Biophotonics</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>Kimberly Ashman; Brian Summa; Sharon Fox; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Super-Resolution and Focus Recovery in Whole Slide Images Using CycleGAN</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Optica Biophotonics</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Huimin Zhuge; Kimberly Ashman; Brian Summa; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Interactive WSI Review and Annotation Tracker, and Digital Visualization Tool for Pathologist Diagnosis of Whole Slide Images</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Optica Biophotonics</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>Huimin Zhuge; David Manthey; Kimberly Ashman; Brian Summa; Roni Choudhury; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>A Camera-Assisted Pathology Microscope to Capture the Lost Data in Clinical Glass Slide Diagnosis</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>bioRxiv</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Kimberly Ashman; Max S. Cooper; Huimin Zhuge; Sharon E. Fox; Jonathan I. Epstein; Carola Wenk; Brian Summa; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Using Morphological Features of Seafloor Sidescans to Predict Biological Presence</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>AGU</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>Heather L. Holcomb; Cooper Maira; Brian Summa; Yizhaq Makovsky; Cynthia J. Ebinger</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Towards Automatic Classification of Synthetic Aperture Sonar Images: Levant Margin Case Study</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>AGU</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Heather L. Holcomb; Cooper Maira; Cody Licorish; Yizhaq Makovsky; Brian Summa; Cynthia Ebinger</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>User-Interactive, On-Demand CycleGAN-Based Super Resolution and Focus Recovery on Whole Slide Images</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>WiML</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>Huimin Zhuge; Brian Summa; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Fast Searching in Scientific Datasets Using Topological Similarity</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>CRA-WP Grad Cohort</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Yu Qin; Brittany Terese Fasy; Carola Wenk; Brian Summa</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Image-Assisted Analysis of Pathologist Slide Review as a Means of Informing Optimal Digital Slide Acquisition Strategies</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>SPIE</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>Short Paper</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>Kimberly Ashman; Brian Summa; Sharon E. Fox; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Comparing Distance Metrics on Vectorized Persistence Summaries</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>NeurIPS TDA Workshop</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>Workshop Paper</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>Brittany Terese Fasy; Yu Qin; Brian Summa; Carola Wenk</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Multiscale 3-Dimensional Pathology Findings of COVID-19 Diseased Lung Using High-Resolution Cleared Tissue Microscopy</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>bioRxiv</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Guang Li; Sharon E. Fox; Brian Summa; Bihe Hu; Carola Wenk; Aibek Akmatbekov; Jack L. Harbert; Richard S. Vander Heide; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Assessment of Sampling Adequacy Using Persistent Homology for the Evaluation of Heterogeneity in 3D Histology Acquired through Inverted Selective Plane Illumination Microscopy (iSPIM)</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>SPIE</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>Short Paper</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>Peter Lawson; Bihe Hu; Brittany Terese Fasy; Brian Summa; Carola Wenk; J. Quincy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Flexible Live-Wire: Image Segmentation with Floating Anchors</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>CGF</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>Journal Article</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>Brian Summa; Noura Faraj; Cody Licorish; Valerio Pascucci</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Visualizing the Uncertainty of Graph-Based 2D Segmentation with Min-Path Stability</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>2017</v>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>CGF</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>Journal Article</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>Brian Summa; Julien Tierny; Valerio Pascucci</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Interactive Scripting for Analysis and Visualization of Arbitrarily Large, Disparately Located Climate Data Ensembles Using a Progressive Runtime Server</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>2017</v>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>AGU</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>Brian Summa; Cameron Christensen; Giorgio Scorzelli; Ji-Woo Lee; Aniketh Venkat; Peer-Timo Bremer; Valerio Pascucci</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>A Nonlinear Model for Interactive Data Analysis and Visualization and an Implementation Using Progressive Computation for Massive Remote Climate Data Ensembles</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>2017</v>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>AGU</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>Cameron Christensen; Shusen Liu; Giorgio Scorzelli; Ji-Woo Lee; Aniketh Venkat; Brian Summa; Valerio Pascucci</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>The Grassmannian Atlas: A General Framework for Exploring Linear Projections of High-Dimensional Data</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>2016</v>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>CGF</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>Journal Article</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Shusen Liu; Peer-Timo Bremer; Jayaraman J. Thiagarajan; Bei Wang; Brian Summa; Valerio Pascucci</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>A Scalable Cyberinfrastructure for Interactive Visualization of Terascale Microscopy Data</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>2016</v>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>NYSDS</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>Full Paper</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>Aniketh Venkat; Cameron Christensen; Attila Gyulassy; Brian Summa; Frederick Federer; Alessandra Angelucci; Valerio Pascucci</t>
+        </is>
+      </c>
+      <c r="T87" s="3" t="inlineStr">
+        <is>
+          <t>PubMed: https://pubmed.ncbi.nlm.nih.gov/28638896/</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:T37"/>
@@ -7006,7 +7865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7674,17 +8533,17 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>MAGIC-SCAN: Machine-Learning Assisted Gigantic Image Cancer Margin Scanner</t>
+          <t>MAGIC-SCAN: Machine-Learning Assisted Gigantic-Image Cancer Margin Scanner</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Co-lead</t>
+          <t>Co-PI</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ARPA-H (Precision Surgical Interventions)</t>
+          <t>ARPA-H</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
@@ -7694,10 +8553,8 @@
         <v>2029</v>
       </c>
       <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Up to $22.9M</t>
-        </is>
+      <c r="H17" s="3" t="n">
+        <v>23437420</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
@@ -7711,7 +8568,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Led by Quincy Brown (BME). End year assumes five years.</t>
+          <t>Total is $22,937,420 plus a $500,000 supplement. Award D24AC00338 (Precision Surgical Interventions). PI: J. Quincy Brown. From Brian's CV (Oct 2026).</t>
         </is>
       </c>
     </row>
@@ -7906,27 +8763,27 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>PathCAM: Connecting the Digital Data Pipeline in Diagnostic Pathology with Onboard-Camera Variable Resolution Slide Imaging</t>
+          <t>PathCAM: Repairing the Digital Data Pipeline in Diagnostic Pathology with Onboard-Camera Variable Resolution Slide Imaging</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Co-I</t>
+          <t>Multi-PI</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>NIH (NIGMS R01GM143789)</t>
+          <t>NIH</t>
         </is>
       </c>
       <c r="E23" s="3" t="n">
         <v>2022</v>
       </c>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>$416K in FY2025</t>
-        </is>
+      <c r="F23" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>1696789</v>
       </c>
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
@@ -7937,7 +8794,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>FY2025 amount from NIH RePORTER via ConductScience; check role, years, and total with Brian.</t>
+          <t>Award R01GM143789. Multi-PI with J. Quincy Brown. From Brian's CV (Oct 2026).</t>
         </is>
       </c>
     </row>
@@ -7996,7 +8853,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Early Career Award: Formalizing, Searching, and Streaming Massive Scientific Data</t>
+          <t>Efficient and Accessible Interactive Visual Analytics of Exascale Scientific Data</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -8006,7 +8863,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>U.S. Department of Energy (Office of Science Early Career Research Program)</t>
+          <t>U.S. Department of Energy</t>
         </is>
       </c>
       <c r="E25" s="3" t="n">
@@ -8030,7 +8887,235 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Title paraphrased from the Tulane news story; replace with the official award title.</t>
+          <t>Early Career Research Program, award DE-SC0022873. From Brian's CV (Oct 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Safe, Sustainable, and Resilient Development of Offshore Reservoirs and Natural Gas Upgrading through Innovative Science and Technology (GoMed Consortium)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Senior Personnel</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-Israel Center of Excellence in Energy, Engineering and Water</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>10302000</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>PI: Shantz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>QuBBD: Quantifying Morphologic Phenotypes in Prostate Cancer, Developing Topological Descriptors for Machine Learning Algorithms</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Co-PI</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>NSF/NIH</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>2016</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>479293</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>899999</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nsf.gov/awardsearch/showAward?AWD_ID=1664848</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>imaging</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Award 1664848. PI: Carola Wenk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>EAGER: Scalable, Content-Based, Domain-Agnostic Search of Scientific Data through Concise Topological Representations</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>180000</v>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nsf.gov/awardsearch/showAward?AWD_ID=2136744</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Award 2136744.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>CRII: CHS: Scalable Interactive Image Segmentation through Hierarchical, Query-Driven Processing</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>2016</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>126962</v>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nsf.gov/awardsearch/showAward?AWD_ID=1657020</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Award 1657020.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>IUCRC Planning Grant: Tulane Center for Applied Artificial Intelligence (CAAI)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Co-PI</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>19999</v>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nsf.gov/awardsearch/showAward?AWD_ID=2137285</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Award 2137285. PI: Aron Culotta.</t>
         </is>
       </c>
     </row>
@@ -8051,7 +9136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8903,7 +9988,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Demi Qin and Brian Summa presented merge tree neural networks for rapid topological comparison at IEEE VIS 2024 (published in TVCG).</t>
+          <t>Demi Qin and Brian Summa won a Best Paper Award at IEEE VIS 2024 for merge tree neural networks, a fast way to compare topological structure in scientific data.</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
@@ -8912,7 +9997,7 @@
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2404.05879</t>
+          <t>https://doi.org/10.1109/TVCG.2024.3456395</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -9562,11 +10647,11 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Fangzheng Wu and Brian Summa released a series of preprints on reading and steering the internal states of diffusion transformers and language models.</t>
+          <t>Papers by Fangzheng Wu and Brian Summa were accepted to ICML 2026, EMNLP 2026, and NeurIPS 2026 (two papers), on diffusion models, language model fine-tuning, and reinforcement learning.</t>
         </is>
       </c>
       <c r="D47" s="6" t="n">
-        <v>46152</v>
+        <v>2026</v>
       </c>
       <c r="E47" s="3" t="n"/>
       <c r="F47" s="3" t="inlineStr">
@@ -9574,7 +10659,11 @@
           <t>https://www.alphaxiv.org/@brian-summa</t>
         </is>
       </c>
-      <c r="J47" s="3" t="n"/>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>From Brian's CV (Oct 2026); acceptance months not listed.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -9681,7 +10770,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Paper led by Cooper Maira on ambient, real-time digitization of glass slide microscopy published in Nature Communications.</t>
+          <t>HistoCAM, led by Cooper Maira, was published in Nature Communications. It digitizes glass slide microscopy in real time as pathologists work, a step toward AI at the microscope.</t>
         </is>
       </c>
       <c r="D52" s="3" t="n">
@@ -9728,6 +10817,51 @@
         <is>
           <t>Date from the arXiv IDs (Jun to Sep 2026).</t>
         </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Brian Summa spoke on AI-powered imaging technology for cancer detection in the AI4HealthOutcomes webinar series.</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="n">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Brian Summa received the Tulane School of Science and Engineering Collaborative Team Award and a Tulane Medicine and SSE Synergy Large Grant Award.</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Brian Summa received the IEEE Computer Society Distinguished Service Award for serving as General Chair of IEEE VIS 2021.</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>2022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Conference news, grant pin, and funder name
- Replace the preprints news item with a pinned item on ASSETS 2026
  (Porto, Oct 25-28) and IEEE VIS 2026 (Boston, Nov 9-13) papers
- KeySI is in the IEEE VIS 2026 program
- Add a Pin? column to Grants; pinned grants always show in the first
  five. Pin the NSF civic AI award
- Shorten the GoMed funder to Center of Excellence in Energy,
  Engineering and Water

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nn3skUUzonfjGHPGXscANL
</commit_message>
<xml_diff>
--- a/content/hcc-content.xlsx
+++ b/content/hcc-content.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Students'!$A$1:$O$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Projects'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Papers'!$A$1:$T$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Grants'!$A$1:$K$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Grants'!$A$1:$L$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'News'!$A$1:$J$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Coauthors'!$A$1:$B$44</definedName>
   </definedNames>
@@ -6829,14 +6829,10 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>arXiv</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>Preprint</t>
-        </is>
-      </c>
+          <t>IEEE VIS</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="n"/>
       <c r="H60" s="3" t="inlineStr">
         <is>
           <t>Yan Zhu; Yongbo Chen; Rebecca Faust</t>
@@ -6847,7 +6843,11 @@
           <t>https://arxiv.org/abs/2607.20556</t>
         </is>
       </c>
-      <c r="J60" s="3" t="n"/>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>https://ieeevis.org/year/2026/program/paper/b0f509c7-33eb-4c67-a0cb-a41d7982b2c9/</t>
+        </is>
+      </c>
       <c r="Q60" s="3" t="n"/>
       <c r="T60" s="3" t="n"/>
     </row>
@@ -7865,7 +7865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7879,6 +7879,7 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7937,6 +7938,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Pin?</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -7982,6 +7988,11 @@
         </is>
       </c>
       <c r="K2" s="3" t="n"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -8909,7 +8920,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>U.S.-Israel Center of Excellence in Energy, Engineering and Water</t>
+          <t>Center of Excellence in Energy, Engineering and Water</t>
         </is>
       </c>
       <c r="E26" s="3" t="n">
@@ -8928,7 +8939,7 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>PI: Shantz.</t>
+          <t>U.S.-Israel Center of Excellence in Energy, Engineering and Water. PI: Shantz.</t>
         </is>
       </c>
     </row>
@@ -9120,7 +9131,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K24"/>
+  <autoFilter ref="A1:L30"/>
   <dataValidations count="1">
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"sign,reading,civic,accessviz,scripts,semantic,imaging,topology"</formula1>
@@ -10796,26 +10807,35 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Rebecca, Yongbo, Yan</t>
+          <t>Saad, Rebecca, Chaelin, Yan, Yongbo</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>PhD students Yongbo Chen and Yan Zhu shared new preprints on visualization for debugging data-intensive programs, tuning text embeddings with human feedback (KeySI), and object-level evidence in vision-language models (ProtoLIP).</t>
+          <t>The HCC Group will be at ASSETS 2026 in Porto (October 25–28) and IEEE VIS 2026 in Boston (November 9–13).</t>
         </is>
       </c>
       <c r="D53" s="6" t="n">
-        <v>46266</v>
-      </c>
-      <c r="E53" s="3" t="n"/>
+        <v>46315</v>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>At ASSETS: a scoping review of accessibility research on data visualization by Saad Hassan, Areen Khalaila, and Rebecca Faust, and Chaelin Kim’s ASL video comprehension tool, presented as a paper and a demo. At VIS: KeySI, a framework for tuning text embeddings with human feedback by Yan Zhu, Yongbo Chen, and Rebecca Faust, and a full paper with Rebecca Faust on spatial visual analytics for verifying multi-document summaries.</t>
+        </is>
+      </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2606.30884</t>
+          <t>https://ieeevis.org/year/2026/program/papers/</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>https://assets26.sigaccess.org/</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>Date from the arXiv IDs (Jun to Sep 2026).</t>
+          <t>Conference dates from assets26.sigaccess.org and ieeevis.org (checked Oct 20, 2026).</t>
         </is>
       </c>
     </row>

</xml_diff>